<commit_message>
Update Project5 & 3
</commit_message>
<xml_diff>
--- a/web/templates/Project5/David_version/03_rawPCBmass_PUF.xlsx
+++ b/web/templates/Project5/David_version/03_rawPCBmass_PUF.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\haixi\Documents\DataHarmonizerDevelop\web\templates\Project5\David\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\haixi\Documents\DataHarmonizerDevelop\web\templates\Project5\David_version\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{552D746C-587F-41FC-B28F-4BFDC3C15D6C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DC435B79-E881-4FED-999B-427334FA409F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="33480" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{D186E85A-2681-487D-9322-615EB35A29E6}"/>
+    <workbookView xWindow="-22510" yWindow="-110" windowWidth="22620" windowHeight="13500" xr2:uid="{D186E85A-2681-487D-9322-615EB35A29E6}"/>
   </bookViews>
   <sheets>
     <sheet name="03_rawPCBmass_PUF" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1700" uniqueCount="379">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1700" uniqueCount="380">
   <si>
     <t>percent_biochar</t>
   </si>
@@ -1175,6 +1175,9 @@
   <si>
     <t>David_07</t>
   </si>
+  <si>
+    <t>PCB141</t>
+  </si>
 </sst>
 </file>
 
@@ -1553,34 +1556,34 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{28E26675-B79A-4BD8-A3A7-77E75FF14E30}">
   <dimension ref="A1:GA115"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="10.08984375" customWidth="1"/>
-    <col min="2" max="2" width="15.6328125" customWidth="1"/>
-    <col min="4" max="4" width="18.36328125" customWidth="1"/>
-    <col min="5" max="5" width="15.453125" customWidth="1"/>
-    <col min="49" max="49" width="11.54296875" customWidth="1"/>
-    <col min="62" max="62" width="10.90625" customWidth="1"/>
-    <col min="64" max="64" width="14.1796875" customWidth="1"/>
-    <col min="80" max="80" width="10.453125" customWidth="1"/>
-    <col min="81" max="81" width="15.90625" customWidth="1"/>
-    <col min="82" max="82" width="10.81640625" customWidth="1"/>
-    <col min="85" max="85" width="13.54296875" customWidth="1"/>
-    <col min="88" max="88" width="10.08984375" customWidth="1"/>
-    <col min="100" max="100" width="11.36328125" customWidth="1"/>
-    <col min="114" max="114" width="11.36328125" customWidth="1"/>
-    <col min="115" max="115" width="14.453125" customWidth="1"/>
-    <col min="121" max="121" width="10.81640625" customWidth="1"/>
-    <col min="124" max="124" width="11.1796875" customWidth="1"/>
-    <col min="131" max="131" width="10.90625" customWidth="1"/>
-    <col min="135" max="135" width="10.6328125" customWidth="1"/>
-    <col min="138" max="138" width="10.81640625" customWidth="1"/>
-    <col min="149" max="149" width="11.1796875" customWidth="1"/>
-    <col min="157" max="157" width="11.08984375" customWidth="1"/>
-    <col min="174" max="174" width="10.6328125" customWidth="1"/>
+    <col min="1" max="1" width="10.140625" customWidth="1"/>
+    <col min="2" max="2" width="15.5703125" customWidth="1"/>
+    <col min="4" max="4" width="18.42578125" customWidth="1"/>
+    <col min="5" max="5" width="15.42578125" customWidth="1"/>
+    <col min="49" max="49" width="11.5703125" customWidth="1"/>
+    <col min="62" max="62" width="10.85546875" customWidth="1"/>
+    <col min="64" max="64" width="14.140625" customWidth="1"/>
+    <col min="80" max="80" width="10.42578125" customWidth="1"/>
+    <col min="81" max="81" width="15.85546875" customWidth="1"/>
+    <col min="82" max="82" width="10.85546875" customWidth="1"/>
+    <col min="85" max="85" width="13.5703125" customWidth="1"/>
+    <col min="88" max="88" width="10.140625" customWidth="1"/>
+    <col min="100" max="100" width="11.42578125" customWidth="1"/>
+    <col min="114" max="114" width="11.42578125" customWidth="1"/>
+    <col min="115" max="115" width="14.42578125" customWidth="1"/>
+    <col min="121" max="121" width="10.85546875" customWidth="1"/>
+    <col min="124" max="124" width="11.140625" customWidth="1"/>
+    <col min="131" max="131" width="10.85546875" customWidth="1"/>
+    <col min="135" max="135" width="10.5703125" customWidth="1"/>
+    <col min="138" max="138" width="10.85546875" customWidth="1"/>
+    <col min="149" max="149" width="11.140625" customWidth="1"/>
+    <col min="157" max="157" width="11.140625" customWidth="1"/>
+    <col min="174" max="174" width="10.5703125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:183" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:183" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>13</v>
       </c>
@@ -1954,7 +1957,7 @@
         <v>131</v>
       </c>
       <c r="DU1" t="s">
-        <v>4</v>
+        <v>379</v>
       </c>
       <c r="DV1" t="s">
         <v>132</v>
@@ -2131,7 +2134,7 @@
         <v>189</v>
       </c>
     </row>
-    <row r="2" spans="1:183" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:183" x14ac:dyDescent="0.25">
       <c r="B2" t="s">
         <v>5</v>
       </c>
@@ -2673,7 +2676,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:183" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:183" x14ac:dyDescent="0.25">
       <c r="B3" t="s">
         <v>5</v>
       </c>
@@ -3212,7 +3215,7 @@
         <v>0.11955788198998803</v>
       </c>
     </row>
-    <row r="4" spans="1:183" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:183" x14ac:dyDescent="0.25">
       <c r="B4" t="s">
         <v>5</v>
       </c>
@@ -3754,7 +3757,7 @@
         <v>0.10329167125082921</v>
       </c>
     </row>
-    <row r="5" spans="1:183" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:183" x14ac:dyDescent="0.25">
       <c r="B5" t="s">
         <v>5</v>
       </c>
@@ -4296,7 +4299,7 @@
         <v>9.2278904908334375E-2</v>
       </c>
     </row>
-    <row r="6" spans="1:183" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:183" x14ac:dyDescent="0.25">
       <c r="B6" t="s">
         <v>5</v>
       </c>
@@ -4838,7 +4841,7 @@
         <v>0.12028613842922463</v>
       </c>
     </row>
-    <row r="7" spans="1:183" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:183" x14ac:dyDescent="0.25">
       <c r="B7" t="s">
         <v>5</v>
       </c>
@@ -5380,7 +5383,7 @@
         <v>9.7985276949678138E-2</v>
       </c>
     </row>
-    <row r="8" spans="1:183" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:183" x14ac:dyDescent="0.25">
       <c r="B8" t="s">
         <v>5</v>
       </c>
@@ -5922,7 +5925,7 @@
         <v>0.10017838570485754</v>
       </c>
     </row>
-    <row r="9" spans="1:183" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:183" x14ac:dyDescent="0.25">
       <c r="B9" t="s">
         <v>5</v>
       </c>
@@ -6464,7 +6467,7 @@
         <v>0.108643418088442</v>
       </c>
     </row>
-    <row r="10" spans="1:183" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:183" x14ac:dyDescent="0.25">
       <c r="B10" t="s">
         <v>5</v>
       </c>
@@ -7006,7 +7009,7 @@
         <v>0.10093033384117338</v>
       </c>
     </row>
-    <row r="11" spans="1:183" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:183" x14ac:dyDescent="0.25">
       <c r="B11" t="s">
         <v>5</v>
       </c>
@@ -7548,7 +7551,7 @@
         <v>9.3552850268661503E-2</v>
       </c>
     </row>
-    <row r="12" spans="1:183" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:183" x14ac:dyDescent="0.25">
       <c r="B12" t="s">
         <v>5</v>
       </c>
@@ -8090,7 +8093,7 @@
         <v>8.6014833938643454E-2</v>
       </c>
     </row>
-    <row r="13" spans="1:183" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:183" x14ac:dyDescent="0.25">
       <c r="B13" t="s">
         <v>5</v>
       </c>
@@ -8632,7 +8635,7 @@
         <v>0.10418063119092062</v>
       </c>
     </row>
-    <row r="14" spans="1:183" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:183" x14ac:dyDescent="0.25">
       <c r="B14" t="s">
         <v>5</v>
       </c>
@@ -9174,7 +9177,7 @@
         <v>0.11687301835756347</v>
       </c>
     </row>
-    <row r="15" spans="1:183" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:183" x14ac:dyDescent="0.25">
       <c r="B15" t="s">
         <v>5</v>
       </c>
@@ -9716,7 +9719,7 @@
         <v>0.10100603699084823</v>
       </c>
     </row>
-    <row r="16" spans="1:183" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:183" x14ac:dyDescent="0.25">
       <c r="B16" t="s">
         <v>5</v>
       </c>
@@ -10258,7 +10261,7 @@
         <v>0.11328940165098825</v>
       </c>
     </row>
-    <row r="17" spans="2:181" x14ac:dyDescent="0.35">
+    <row r="17" spans="2:181" x14ac:dyDescent="0.25">
       <c r="B17" t="s">
         <v>5</v>
       </c>
@@ -10800,7 +10803,7 @@
         <v>9.4158553883393573E-2</v>
       </c>
     </row>
-    <row r="18" spans="2:181" x14ac:dyDescent="0.35">
+    <row r="18" spans="2:181" x14ac:dyDescent="0.25">
       <c r="B18" t="s">
         <v>5</v>
       </c>
@@ -11342,7 +11345,7 @@
         <v>8.7683109944317481E-2</v>
       </c>
     </row>
-    <row r="19" spans="2:181" x14ac:dyDescent="0.35">
+    <row r="19" spans="2:181" x14ac:dyDescent="0.25">
       <c r="B19" t="s">
         <v>5</v>
       </c>
@@ -11884,7 +11887,7 @@
         <v>0.1205136926275555</v>
       </c>
     </row>
-    <row r="20" spans="2:181" x14ac:dyDescent="0.35">
+    <row r="20" spans="2:181" x14ac:dyDescent="0.25">
       <c r="B20" t="s">
         <v>5</v>
       </c>
@@ -12426,7 +12429,7 @@
         <v>0.10522515599535914</v>
       </c>
     </row>
-    <row r="21" spans="2:181" x14ac:dyDescent="0.35">
+    <row r="21" spans="2:181" x14ac:dyDescent="0.25">
       <c r="B21" t="s">
         <v>5</v>
       </c>
@@ -12968,7 +12971,7 @@
         <v>7.9550627856596917E-2</v>
       </c>
     </row>
-    <row r="22" spans="2:181" x14ac:dyDescent="0.35">
+    <row r="22" spans="2:181" x14ac:dyDescent="0.25">
       <c r="B22" t="s">
         <v>5</v>
       </c>
@@ -13510,7 +13513,7 @@
         <v>0.10092181931098745</v>
       </c>
     </row>
-    <row r="23" spans="2:181" x14ac:dyDescent="0.35">
+    <row r="23" spans="2:181" x14ac:dyDescent="0.25">
       <c r="B23" t="s">
         <v>10</v>
       </c>
@@ -14052,7 +14055,7 @@
         <v>3.0098653903668118E-3</v>
       </c>
     </row>
-    <row r="24" spans="2:181" x14ac:dyDescent="0.35">
+    <row r="24" spans="2:181" x14ac:dyDescent="0.25">
       <c r="B24" t="s">
         <v>10</v>
       </c>
@@ -14594,7 +14597,7 @@
         <v>4.6673465235767602E-3</v>
       </c>
     </row>
-    <row r="25" spans="2:181" x14ac:dyDescent="0.35">
+    <row r="25" spans="2:181" x14ac:dyDescent="0.25">
       <c r="B25" t="s">
         <v>10</v>
       </c>
@@ -15136,7 +15139,7 @@
         <v>4.2737308860793556E-3</v>
       </c>
     </row>
-    <row r="26" spans="2:181" x14ac:dyDescent="0.35">
+    <row r="26" spans="2:181" x14ac:dyDescent="0.25">
       <c r="B26" t="s">
         <v>10</v>
       </c>
@@ -15678,7 +15681,7 @@
         <v>5.2152430154873645E-3</v>
       </c>
     </row>
-    <row r="27" spans="2:181" x14ac:dyDescent="0.35">
+    <row r="27" spans="2:181" x14ac:dyDescent="0.25">
       <c r="B27" t="s">
         <v>10</v>
       </c>
@@ -16220,7 +16223,7 @@
         <v>4.3595635923305504E-3</v>
       </c>
     </row>
-    <row r="28" spans="2:181" x14ac:dyDescent="0.35">
+    <row r="28" spans="2:181" x14ac:dyDescent="0.25">
       <c r="B28" t="s">
         <v>10</v>
       </c>
@@ -16762,7 +16765,7 @@
         <v>5.4336096640223101E-3</v>
       </c>
     </row>
-    <row r="29" spans="2:181" x14ac:dyDescent="0.35">
+    <row r="29" spans="2:181" x14ac:dyDescent="0.25">
       <c r="B29" t="s">
         <v>10</v>
       </c>
@@ -17304,7 +17307,7 @@
         <v>4.9511656769862808E-3</v>
       </c>
     </row>
-    <row r="30" spans="2:181" x14ac:dyDescent="0.35">
+    <row r="30" spans="2:181" x14ac:dyDescent="0.25">
       <c r="B30" t="s">
         <v>10</v>
       </c>
@@ -17846,7 +17849,7 @@
         <v>4.3158350172819611E-3</v>
       </c>
     </row>
-    <row r="31" spans="2:181" x14ac:dyDescent="0.35">
+    <row r="31" spans="2:181" x14ac:dyDescent="0.25">
       <c r="B31" t="s">
         <v>10</v>
       </c>
@@ -18388,7 +18391,7 @@
         <v>4.6668361181313499E-3</v>
       </c>
     </row>
-    <row r="32" spans="2:181" x14ac:dyDescent="0.35">
+    <row r="32" spans="2:181" x14ac:dyDescent="0.25">
       <c r="B32" t="s">
         <v>10</v>
       </c>
@@ -18930,7 +18933,7 @@
         <v>5.3380535181210874E-3</v>
       </c>
     </row>
-    <row r="33" spans="2:181" x14ac:dyDescent="0.35">
+    <row r="33" spans="2:181" x14ac:dyDescent="0.25">
       <c r="B33" t="s">
         <v>10</v>
       </c>
@@ -19472,7 +19475,7 @@
         <v>5.8634460496947939E-3</v>
       </c>
     </row>
-    <row r="34" spans="2:181" x14ac:dyDescent="0.35">
+    <row r="34" spans="2:181" x14ac:dyDescent="0.25">
       <c r="B34" t="s">
         <v>10</v>
       </c>
@@ -20014,7 +20017,7 @@
         <v>4.6606067394770892E-3</v>
       </c>
     </row>
-    <row r="35" spans="2:181" x14ac:dyDescent="0.35">
+    <row r="35" spans="2:181" x14ac:dyDescent="0.25">
       <c r="B35" t="s">
         <v>10</v>
       </c>
@@ -20556,7 +20559,7 @@
         <v>4.9498255674751308E-3</v>
       </c>
     </row>
-    <row r="36" spans="2:181" x14ac:dyDescent="0.35">
+    <row r="36" spans="2:181" x14ac:dyDescent="0.25">
       <c r="B36" t="s">
         <v>10</v>
       </c>
@@ -21098,7 +21101,7 @@
         <v>4.5556525779325398E-3</v>
       </c>
     </row>
-    <row r="37" spans="2:181" x14ac:dyDescent="0.35">
+    <row r="37" spans="2:181" x14ac:dyDescent="0.25">
       <c r="B37" t="s">
         <v>10</v>
       </c>
@@ -21640,7 +21643,7 @@
         <v>5.8066340592319403E-3</v>
       </c>
     </row>
-    <row r="38" spans="2:181" x14ac:dyDescent="0.35">
+    <row r="38" spans="2:181" x14ac:dyDescent="0.25">
       <c r="B38" t="s">
         <v>10</v>
       </c>
@@ -22182,7 +22185,7 @@
         <v>5.2624792988532178E-3</v>
       </c>
     </row>
-    <row r="39" spans="2:181" x14ac:dyDescent="0.35">
+    <row r="39" spans="2:181" x14ac:dyDescent="0.25">
       <c r="B39" t="s">
         <v>10</v>
       </c>
@@ -22724,7 +22727,7 @@
         <v>5.4604811038541012E-3</v>
       </c>
     </row>
-    <row r="40" spans="2:181" x14ac:dyDescent="0.35">
+    <row r="40" spans="2:181" x14ac:dyDescent="0.25">
       <c r="B40" t="s">
         <v>10</v>
       </c>
@@ -23266,7 +23269,7 @@
         <v>6.598720934751617E-3</v>
       </c>
     </row>
-    <row r="41" spans="2:181" x14ac:dyDescent="0.35">
+    <row r="41" spans="2:181" x14ac:dyDescent="0.25">
       <c r="B41" t="s">
         <v>10</v>
       </c>
@@ -23808,7 +23811,7 @@
         <v>5.7536077375787056E-3</v>
       </c>
     </row>
-    <row r="42" spans="2:181" x14ac:dyDescent="0.35">
+    <row r="42" spans="2:181" x14ac:dyDescent="0.25">
       <c r="B42" t="s">
         <v>10</v>
       </c>
@@ -24350,7 +24353,7 @@
         <v>5.3805766385150817E-3</v>
       </c>
     </row>
-    <row r="43" spans="2:181" x14ac:dyDescent="0.35">
+    <row r="43" spans="2:181" x14ac:dyDescent="0.25">
       <c r="B43" t="s">
         <v>10</v>
       </c>
@@ -24892,7 +24895,7 @@
         <v>4.4920417120483426E-3</v>
       </c>
     </row>
-    <row r="44" spans="2:181" x14ac:dyDescent="0.35">
+    <row r="44" spans="2:181" x14ac:dyDescent="0.25">
       <c r="B44" t="s">
         <v>5</v>
       </c>
@@ -25434,7 +25437,7 @@
         <v>6.4826510465640377E-2</v>
       </c>
     </row>
-    <row r="45" spans="2:181" x14ac:dyDescent="0.35">
+    <row r="45" spans="2:181" x14ac:dyDescent="0.25">
       <c r="B45" t="s">
         <v>5</v>
       </c>
@@ -25976,7 +25979,7 @@
         <v>6.734303874755998E-2</v>
       </c>
     </row>
-    <row r="46" spans="2:181" x14ac:dyDescent="0.35">
+    <row r="46" spans="2:181" x14ac:dyDescent="0.25">
       <c r="B46" t="s">
         <v>5</v>
       </c>
@@ -26518,7 +26521,7 @@
         <v>8.805396750048132E-2</v>
       </c>
     </row>
-    <row r="47" spans="2:181" x14ac:dyDescent="0.35">
+    <row r="47" spans="2:181" x14ac:dyDescent="0.25">
       <c r="B47" t="s">
         <v>5</v>
       </c>
@@ -27060,7 +27063,7 @@
         <v>6.2017534526315789E-2</v>
       </c>
     </row>
-    <row r="48" spans="2:181" x14ac:dyDescent="0.35">
+    <row r="48" spans="2:181" x14ac:dyDescent="0.25">
       <c r="B48" t="s">
         <v>5</v>
       </c>
@@ -27602,7 +27605,7 @@
         <v>9.921069259918007E-2</v>
       </c>
     </row>
-    <row r="49" spans="2:181" x14ac:dyDescent="0.35">
+    <row r="49" spans="2:181" x14ac:dyDescent="0.25">
       <c r="B49" t="s">
         <v>5</v>
       </c>
@@ -28144,7 +28147,7 @@
         <v>8.79925962443181E-2</v>
       </c>
     </row>
-    <row r="50" spans="2:181" x14ac:dyDescent="0.35">
+    <row r="50" spans="2:181" x14ac:dyDescent="0.25">
       <c r="B50" t="s">
         <v>5</v>
       </c>
@@ -28686,7 +28689,7 @@
         <v>9.0603646244250782E-2</v>
       </c>
     </row>
-    <row r="51" spans="2:181" x14ac:dyDescent="0.35">
+    <row r="51" spans="2:181" x14ac:dyDescent="0.25">
       <c r="B51" t="s">
         <v>5</v>
       </c>
@@ -29228,7 +29231,7 @@
         <v>6.9147877865697316E-2</v>
       </c>
     </row>
-    <row r="52" spans="2:181" x14ac:dyDescent="0.35">
+    <row r="52" spans="2:181" x14ac:dyDescent="0.25">
       <c r="B52" t="s">
         <v>5</v>
       </c>
@@ -29770,7 +29773,7 @@
         <v>7.8528053646848742E-2</v>
       </c>
     </row>
-    <row r="53" spans="2:181" x14ac:dyDescent="0.35">
+    <row r="53" spans="2:181" x14ac:dyDescent="0.25">
       <c r="B53" t="s">
         <v>5</v>
       </c>
@@ -30312,7 +30315,7 @@
         <v>6.9055021578371484E-2</v>
       </c>
     </row>
-    <row r="54" spans="2:181" x14ac:dyDescent="0.35">
+    <row r="54" spans="2:181" x14ac:dyDescent="0.25">
       <c r="B54" t="s">
         <v>5</v>
       </c>
@@ -30854,7 +30857,7 @@
         <v>0.13964264318758066</v>
       </c>
     </row>
-    <row r="55" spans="2:181" x14ac:dyDescent="0.35">
+    <row r="55" spans="2:181" x14ac:dyDescent="0.25">
       <c r="B55" t="s">
         <v>5</v>
       </c>
@@ -31396,7 +31399,7 @@
         <v>0.10529422700366056</v>
       </c>
     </row>
-    <row r="56" spans="2:181" x14ac:dyDescent="0.35">
+    <row r="56" spans="2:181" x14ac:dyDescent="0.25">
       <c r="B56" t="s">
         <v>5</v>
       </c>
@@ -31938,7 +31941,7 @@
         <v>0.10665414010784678</v>
       </c>
     </row>
-    <row r="57" spans="2:181" x14ac:dyDescent="0.35">
+    <row r="57" spans="2:181" x14ac:dyDescent="0.25">
       <c r="B57" t="s">
         <v>5</v>
       </c>
@@ -32480,7 +32483,7 @@
         <v>9.1026951203902293E-2</v>
       </c>
     </row>
-    <row r="58" spans="2:181" x14ac:dyDescent="0.35">
+    <row r="58" spans="2:181" x14ac:dyDescent="0.25">
       <c r="B58" t="s">
         <v>5</v>
       </c>
@@ -33022,7 +33025,7 @@
         <v>8.647548318780611E-2</v>
       </c>
     </row>
-    <row r="59" spans="2:181" x14ac:dyDescent="0.35">
+    <row r="59" spans="2:181" x14ac:dyDescent="0.25">
       <c r="B59" t="s">
         <v>5</v>
       </c>
@@ -33564,7 +33567,7 @@
         <v>8.1948485585723291E-2</v>
       </c>
     </row>
-    <row r="60" spans="2:181" x14ac:dyDescent="0.35">
+    <row r="60" spans="2:181" x14ac:dyDescent="0.25">
       <c r="B60" t="s">
         <v>5</v>
       </c>
@@ -34106,7 +34109,7 @@
         <v>0.10546770631485064</v>
       </c>
     </row>
-    <row r="61" spans="2:181" x14ac:dyDescent="0.35">
+    <row r="61" spans="2:181" x14ac:dyDescent="0.25">
       <c r="B61" t="s">
         <v>5</v>
       </c>
@@ -34648,7 +34651,7 @@
         <v>7.5654071341648046E-2</v>
       </c>
     </row>
-    <row r="62" spans="2:181" x14ac:dyDescent="0.35">
+    <row r="62" spans="2:181" x14ac:dyDescent="0.25">
       <c r="B62" t="s">
         <v>5</v>
       </c>
@@ -35190,7 +35193,7 @@
         <v>0.10179487491812268</v>
       </c>
     </row>
-    <row r="63" spans="2:181" x14ac:dyDescent="0.35">
+    <row r="63" spans="2:181" x14ac:dyDescent="0.25">
       <c r="B63" t="s">
         <v>5</v>
       </c>
@@ -35732,7 +35735,7 @@
         <v>0.10682423991093562</v>
       </c>
     </row>
-    <row r="64" spans="2:181" x14ac:dyDescent="0.35">
+    <row r="64" spans="2:181" x14ac:dyDescent="0.25">
       <c r="B64" t="s">
         <v>5</v>
       </c>
@@ -36274,7 +36277,7 @@
         <v>0.10786376301582896</v>
       </c>
     </row>
-    <row r="65" spans="2:181" x14ac:dyDescent="0.35">
+    <row r="65" spans="2:181" x14ac:dyDescent="0.25">
       <c r="B65" t="s">
         <v>5</v>
       </c>
@@ -36816,7 +36819,7 @@
         <v>0.11327923912943738</v>
       </c>
     </row>
-    <row r="66" spans="2:181" x14ac:dyDescent="0.35">
+    <row r="66" spans="2:181" x14ac:dyDescent="0.25">
       <c r="B66" t="s">
         <v>5</v>
       </c>
@@ -37358,7 +37361,7 @@
         <v>0.10351893392686821</v>
       </c>
     </row>
-    <row r="67" spans="2:181" x14ac:dyDescent="0.35">
+    <row r="67" spans="2:181" x14ac:dyDescent="0.25">
       <c r="B67" t="s">
         <v>5</v>
       </c>
@@ -37900,7 +37903,7 @@
         <v>0.10830373800362383</v>
       </c>
     </row>
-    <row r="68" spans="2:181" x14ac:dyDescent="0.35">
+    <row r="68" spans="2:181" x14ac:dyDescent="0.25">
       <c r="B68" t="s">
         <v>5</v>
       </c>
@@ -38442,7 +38445,7 @@
         <v>0.11253413643600441</v>
       </c>
     </row>
-    <row r="69" spans="2:181" x14ac:dyDescent="0.35">
+    <row r="69" spans="2:181" x14ac:dyDescent="0.25">
       <c r="B69" t="s">
         <v>5</v>
       </c>
@@ -38984,7 +38987,7 @@
         <v>0.11093882599317245</v>
       </c>
     </row>
-    <row r="70" spans="2:181" x14ac:dyDescent="0.35">
+    <row r="70" spans="2:181" x14ac:dyDescent="0.25">
       <c r="B70" t="s">
         <v>5</v>
       </c>
@@ -39526,7 +39529,7 @@
         <v>9.7500540445111403E-2</v>
       </c>
     </row>
-    <row r="71" spans="2:181" x14ac:dyDescent="0.35">
+    <row r="71" spans="2:181" x14ac:dyDescent="0.25">
       <c r="B71" t="s">
         <v>5</v>
       </c>
@@ -40068,7 +40071,7 @@
         <v>0.11091983039816043</v>
       </c>
     </row>
-    <row r="72" spans="2:181" x14ac:dyDescent="0.35">
+    <row r="72" spans="2:181" x14ac:dyDescent="0.25">
       <c r="B72" t="s">
         <v>5</v>
       </c>
@@ -40610,7 +40613,7 @@
         <v>0.10615568446871926</v>
       </c>
     </row>
-    <row r="73" spans="2:181" x14ac:dyDescent="0.35">
+    <row r="73" spans="2:181" x14ac:dyDescent="0.25">
       <c r="B73" t="s">
         <v>5</v>
       </c>
@@ -41152,7 +41155,7 @@
         <v>0.11699080539725204</v>
       </c>
     </row>
-    <row r="74" spans="2:181" x14ac:dyDescent="0.35">
+    <row r="74" spans="2:181" x14ac:dyDescent="0.25">
       <c r="B74" t="s">
         <v>5</v>
       </c>
@@ -41694,7 +41697,7 @@
         <v>0.1315640699346525</v>
       </c>
     </row>
-    <row r="75" spans="2:181" x14ac:dyDescent="0.35">
+    <row r="75" spans="2:181" x14ac:dyDescent="0.25">
       <c r="B75" t="s">
         <v>5</v>
       </c>
@@ -42236,7 +42239,7 @@
         <v>0.15870324822691015</v>
       </c>
     </row>
-    <row r="76" spans="2:181" x14ac:dyDescent="0.35">
+    <row r="76" spans="2:181" x14ac:dyDescent="0.25">
       <c r="B76" t="s">
         <v>5</v>
       </c>
@@ -42778,7 +42781,7 @@
         <v>0.10797195549675623</v>
       </c>
     </row>
-    <row r="77" spans="2:181" x14ac:dyDescent="0.35">
+    <row r="77" spans="2:181" x14ac:dyDescent="0.25">
       <c r="B77" t="s">
         <v>5</v>
       </c>
@@ -43320,7 +43323,7 @@
         <v>0.11624260249866605</v>
       </c>
     </row>
-    <row r="78" spans="2:181" x14ac:dyDescent="0.35">
+    <row r="78" spans="2:181" x14ac:dyDescent="0.25">
       <c r="B78" t="s">
         <v>5</v>
       </c>
@@ -43862,7 +43865,7 @@
         <v>0.11869685606732593</v>
       </c>
     </row>
-    <row r="79" spans="2:181" x14ac:dyDescent="0.35">
+    <row r="79" spans="2:181" x14ac:dyDescent="0.25">
       <c r="B79" t="s">
         <v>5</v>
       </c>
@@ -44404,7 +44407,7 @@
         <v>0.1214405373130573</v>
       </c>
     </row>
-    <row r="80" spans="2:181" x14ac:dyDescent="0.35">
+    <row r="80" spans="2:181" x14ac:dyDescent="0.25">
       <c r="B80" t="s">
         <v>10</v>
       </c>
@@ -44946,7 +44949,7 @@
         <v>6.5813566951703709E-3</v>
       </c>
     </row>
-    <row r="81" spans="2:181" x14ac:dyDescent="0.35">
+    <row r="81" spans="2:181" x14ac:dyDescent="0.25">
       <c r="B81" t="s">
         <v>10</v>
       </c>
@@ -45488,7 +45491,7 @@
         <v>6.6858953168688418E-3</v>
       </c>
     </row>
-    <row r="82" spans="2:181" x14ac:dyDescent="0.35">
+    <row r="82" spans="2:181" x14ac:dyDescent="0.25">
       <c r="B82" t="s">
         <v>10</v>
       </c>
@@ -46030,7 +46033,7 @@
         <v>6.6243781594205438E-3</v>
       </c>
     </row>
-    <row r="83" spans="2:181" x14ac:dyDescent="0.35">
+    <row r="83" spans="2:181" x14ac:dyDescent="0.25">
       <c r="B83" t="s">
         <v>10</v>
       </c>
@@ -46572,7 +46575,7 @@
         <v>5.0106098881415916E-3</v>
       </c>
     </row>
-    <row r="84" spans="2:181" x14ac:dyDescent="0.35">
+    <row r="84" spans="2:181" x14ac:dyDescent="0.25">
       <c r="B84" t="s">
         <v>10</v>
       </c>
@@ -47114,7 +47117,7 @@
         <v>5.2708573078878874E-3</v>
       </c>
     </row>
-    <row r="85" spans="2:181" x14ac:dyDescent="0.35">
+    <row r="85" spans="2:181" x14ac:dyDescent="0.25">
       <c r="B85" t="s">
         <v>10</v>
       </c>
@@ -47656,7 +47659,7 @@
         <v>5.014977417833506E-3</v>
       </c>
     </row>
-    <row r="86" spans="2:181" x14ac:dyDescent="0.35">
+    <row r="86" spans="2:181" x14ac:dyDescent="0.25">
       <c r="B86" t="s">
         <v>10</v>
       </c>
@@ -48198,7 +48201,7 @@
         <v>4.9617564369556387E-3</v>
       </c>
     </row>
-    <row r="87" spans="2:181" x14ac:dyDescent="0.35">
+    <row r="87" spans="2:181" x14ac:dyDescent="0.25">
       <c r="B87" t="s">
         <v>10</v>
       </c>
@@ -48740,7 +48743,7 @@
         <v>8.138283488086524E-3</v>
       </c>
     </row>
-    <row r="88" spans="2:181" x14ac:dyDescent="0.35">
+    <row r="88" spans="2:181" x14ac:dyDescent="0.25">
       <c r="B88" t="s">
         <v>10</v>
       </c>
@@ -49282,7 +49285,7 @@
         <v>6.8851239075057649E-3</v>
       </c>
     </row>
-    <row r="89" spans="2:181" x14ac:dyDescent="0.35">
+    <row r="89" spans="2:181" x14ac:dyDescent="0.25">
       <c r="B89" t="s">
         <v>10</v>
       </c>
@@ -49824,7 +49827,7 @@
         <v>9.0361490924004209E-3</v>
       </c>
     </row>
-    <row r="90" spans="2:181" x14ac:dyDescent="0.35">
+    <row r="90" spans="2:181" x14ac:dyDescent="0.25">
       <c r="B90" t="s">
         <v>10</v>
       </c>
@@ -50366,7 +50369,7 @@
         <v>7.5922220251629135E-3</v>
       </c>
     </row>
-    <row r="91" spans="2:181" x14ac:dyDescent="0.35">
+    <row r="91" spans="2:181" x14ac:dyDescent="0.25">
       <c r="B91" t="s">
         <v>10</v>
       </c>
@@ -50908,7 +50911,7 @@
         <v>5.0924397631352692E-3</v>
       </c>
     </row>
-    <row r="92" spans="2:181" x14ac:dyDescent="0.35">
+    <row r="92" spans="2:181" x14ac:dyDescent="0.25">
       <c r="B92" t="s">
         <v>10</v>
       </c>
@@ -51450,7 +51453,7 @@
         <v>6.8359457483283129E-3</v>
       </c>
     </row>
-    <row r="93" spans="2:181" x14ac:dyDescent="0.35">
+    <row r="93" spans="2:181" x14ac:dyDescent="0.25">
       <c r="B93" t="s">
         <v>10</v>
       </c>
@@ -51992,7 +51995,7 @@
         <v>5.7133333268304777E-3</v>
       </c>
     </row>
-    <row r="94" spans="2:181" x14ac:dyDescent="0.35">
+    <row r="94" spans="2:181" x14ac:dyDescent="0.25">
       <c r="B94" t="s">
         <v>10</v>
       </c>
@@ -52534,7 +52537,7 @@
         <v>4.9169411181819696E-3</v>
       </c>
     </row>
-    <row r="95" spans="2:181" x14ac:dyDescent="0.35">
+    <row r="95" spans="2:181" x14ac:dyDescent="0.25">
       <c r="B95" t="s">
         <v>10</v>
       </c>
@@ -52557,7 +52560,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="96" spans="2:181" x14ac:dyDescent="0.35">
+    <row r="96" spans="2:181" x14ac:dyDescent="0.25">
       <c r="B96" t="s">
         <v>10</v>
       </c>
@@ -53099,7 +53102,7 @@
         <v>5.0266996956255293E-3</v>
       </c>
     </row>
-    <row r="97" spans="2:181" x14ac:dyDescent="0.35">
+    <row r="97" spans="2:181" x14ac:dyDescent="0.25">
       <c r="B97" t="s">
         <v>10</v>
       </c>
@@ -53641,7 +53644,7 @@
         <v>5.1104845366235644E-3</v>
       </c>
     </row>
-    <row r="98" spans="2:181" x14ac:dyDescent="0.35">
+    <row r="98" spans="2:181" x14ac:dyDescent="0.25">
       <c r="B98" t="s">
         <v>10</v>
       </c>
@@ -54183,7 +54186,7 @@
         <v>5.2563081139359894E-3</v>
       </c>
     </row>
-    <row r="99" spans="2:181" x14ac:dyDescent="0.35">
+    <row r="99" spans="2:181" x14ac:dyDescent="0.25">
       <c r="B99" t="s">
         <v>10</v>
       </c>
@@ -54725,7 +54728,7 @@
         <v>6.5051398079765078E-3</v>
       </c>
     </row>
-    <row r="100" spans="2:181" x14ac:dyDescent="0.35">
+    <row r="100" spans="2:181" x14ac:dyDescent="0.25">
       <c r="B100" t="s">
         <v>10</v>
       </c>
@@ -55267,7 +55270,7 @@
         <v>4.2367578240077915E-3</v>
       </c>
     </row>
-    <row r="101" spans="2:181" x14ac:dyDescent="0.35">
+    <row r="101" spans="2:181" x14ac:dyDescent="0.25">
       <c r="B101" t="s">
         <v>10</v>
       </c>
@@ -55809,7 +55812,7 @@
         <v>5.0078668393337133E-3</v>
       </c>
     </row>
-    <row r="102" spans="2:181" x14ac:dyDescent="0.35">
+    <row r="102" spans="2:181" x14ac:dyDescent="0.25">
       <c r="B102" t="s">
         <v>10</v>
       </c>
@@ -56351,7 +56354,7 @@
         <v>4.6427739703734511E-3</v>
       </c>
     </row>
-    <row r="103" spans="2:181" x14ac:dyDescent="0.35">
+    <row r="103" spans="2:181" x14ac:dyDescent="0.25">
       <c r="B103" t="s">
         <v>10</v>
       </c>
@@ -56893,7 +56896,7 @@
         <v>4.8786742431402913E-3</v>
       </c>
     </row>
-    <row r="104" spans="2:181" x14ac:dyDescent="0.35">
+    <row r="104" spans="2:181" x14ac:dyDescent="0.25">
       <c r="B104" t="s">
         <v>10</v>
       </c>
@@ -57435,7 +57438,7 @@
         <v>5.2374408435720294E-3</v>
       </c>
     </row>
-    <row r="105" spans="2:181" x14ac:dyDescent="0.35">
+    <row r="105" spans="2:181" x14ac:dyDescent="0.25">
       <c r="B105" t="s">
         <v>10</v>
       </c>
@@ -57977,7 +57980,7 @@
         <v>7.3565402501294206E-3</v>
       </c>
     </row>
-    <row r="106" spans="2:181" x14ac:dyDescent="0.35">
+    <row r="106" spans="2:181" x14ac:dyDescent="0.25">
       <c r="B106" t="s">
         <v>10</v>
       </c>
@@ -58519,7 +58522,7 @@
         <v>5.1346716181612777E-3</v>
       </c>
     </row>
-    <row r="107" spans="2:181" x14ac:dyDescent="0.35">
+    <row r="107" spans="2:181" x14ac:dyDescent="0.25">
       <c r="B107" t="s">
         <v>10</v>
       </c>
@@ -59061,7 +59064,7 @@
         <v>1.1408385848245453E-2</v>
       </c>
     </row>
-    <row r="108" spans="2:181" x14ac:dyDescent="0.35">
+    <row r="108" spans="2:181" x14ac:dyDescent="0.25">
       <c r="B108" t="s">
         <v>10</v>
       </c>
@@ -59603,7 +59606,7 @@
         <v>1.1328188985726835E-2</v>
       </c>
     </row>
-    <row r="109" spans="2:181" x14ac:dyDescent="0.35">
+    <row r="109" spans="2:181" x14ac:dyDescent="0.25">
       <c r="B109" t="s">
         <v>10</v>
       </c>
@@ -60145,7 +60148,7 @@
         <v>8.8464370205292558E-3</v>
       </c>
     </row>
-    <row r="110" spans="2:181" x14ac:dyDescent="0.35">
+    <row r="110" spans="2:181" x14ac:dyDescent="0.25">
       <c r="B110" t="s">
         <v>10</v>
       </c>
@@ -60687,7 +60690,7 @@
         <v>6.9282934280876481E-3</v>
       </c>
     </row>
-    <row r="111" spans="2:181" x14ac:dyDescent="0.35">
+    <row r="111" spans="2:181" x14ac:dyDescent="0.25">
       <c r="B111" t="s">
         <v>10</v>
       </c>
@@ -61229,7 +61232,7 @@
         <v>7.2563566640260297E-3</v>
       </c>
     </row>
-    <row r="112" spans="2:181" x14ac:dyDescent="0.35">
+    <row r="112" spans="2:181" x14ac:dyDescent="0.25">
       <c r="B112" t="s">
         <v>10</v>
       </c>
@@ -61771,7 +61774,7 @@
         <v>8.870596879290411E-3</v>
       </c>
     </row>
-    <row r="113" spans="2:181" x14ac:dyDescent="0.35">
+    <row r="113" spans="2:181" x14ac:dyDescent="0.25">
       <c r="B113" t="s">
         <v>10</v>
       </c>
@@ -62313,7 +62316,7 @@
         <v>7.9438753663435072E-3</v>
       </c>
     </row>
-    <row r="114" spans="2:181" x14ac:dyDescent="0.35">
+    <row r="114" spans="2:181" x14ac:dyDescent="0.25">
       <c r="B114" t="s">
         <v>10</v>
       </c>
@@ -62855,7 +62858,7 @@
         <v>8.0685499983665782E-3</v>
       </c>
     </row>
-    <row r="115" spans="2:181" x14ac:dyDescent="0.35">
+    <row r="115" spans="2:181" x14ac:dyDescent="0.25">
       <c r="B115" t="s">
         <v>10</v>
       </c>
@@ -63405,36 +63408,36 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4C21E329-08CE-448A-A06B-F413BC3767B8}">
   <dimension ref="A1:FS10"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="18.6328125" customWidth="1"/>
-    <col min="18" max="18" width="9.26953125" customWidth="1"/>
-    <col min="21" max="21" width="10.81640625" customWidth="1"/>
-    <col min="26" max="26" width="10.36328125" customWidth="1"/>
-    <col min="40" max="40" width="12.1796875" customWidth="1"/>
-    <col min="44" max="44" width="11.36328125" customWidth="1"/>
-    <col min="45" max="45" width="11.08984375" customWidth="1"/>
-    <col min="53" max="53" width="12.54296875" customWidth="1"/>
-    <col min="55" max="55" width="16.26953125" customWidth="1"/>
-    <col min="71" max="71" width="11.90625" customWidth="1"/>
-    <col min="72" max="72" width="17.6328125" customWidth="1"/>
-    <col min="73" max="73" width="11.1796875" customWidth="1"/>
-    <col min="76" max="76" width="14.81640625" customWidth="1"/>
-    <col min="79" max="79" width="10.7265625" customWidth="1"/>
-    <col min="91" max="91" width="11.54296875" customWidth="1"/>
-    <col min="105" max="105" width="13.1796875" customWidth="1"/>
-    <col min="106" max="106" width="15.54296875" customWidth="1"/>
-    <col min="112" max="112" width="11.6328125" customWidth="1"/>
-    <col min="115" max="115" width="11.6328125" customWidth="1"/>
-    <col min="122" max="122" width="11.6328125" customWidth="1"/>
-    <col min="126" max="126" width="11.453125" customWidth="1"/>
-    <col min="129" max="129" width="13.26953125" customWidth="1"/>
-    <col min="140" max="140" width="11.90625" customWidth="1"/>
-    <col min="148" max="148" width="12.36328125" customWidth="1"/>
-    <col min="165" max="165" width="12.1796875" customWidth="1"/>
+    <col min="1" max="1" width="18.5703125" customWidth="1"/>
+    <col min="18" max="18" width="9.28515625" customWidth="1"/>
+    <col min="21" max="21" width="10.85546875" customWidth="1"/>
+    <col min="26" max="26" width="10.42578125" customWidth="1"/>
+    <col min="40" max="40" width="12.140625" customWidth="1"/>
+    <col min="44" max="44" width="11.42578125" customWidth="1"/>
+    <col min="45" max="45" width="11.140625" customWidth="1"/>
+    <col min="53" max="53" width="12.5703125" customWidth="1"/>
+    <col min="55" max="55" width="16.28515625" customWidth="1"/>
+    <col min="71" max="71" width="11.85546875" customWidth="1"/>
+    <col min="72" max="72" width="17.5703125" customWidth="1"/>
+    <col min="73" max="73" width="11.140625" customWidth="1"/>
+    <col min="76" max="76" width="14.85546875" customWidth="1"/>
+    <col min="79" max="79" width="10.7109375" customWidth="1"/>
+    <col min="91" max="91" width="11.5703125" customWidth="1"/>
+    <col min="105" max="105" width="13.140625" customWidth="1"/>
+    <col min="106" max="106" width="15.5703125" customWidth="1"/>
+    <col min="112" max="112" width="11.5703125" customWidth="1"/>
+    <col min="115" max="115" width="11.5703125" customWidth="1"/>
+    <col min="122" max="122" width="11.5703125" customWidth="1"/>
+    <col min="126" max="126" width="11.42578125" customWidth="1"/>
+    <col min="129" max="129" width="13.28515625" customWidth="1"/>
+    <col min="140" max="140" width="11.85546875" customWidth="1"/>
+    <col min="148" max="148" width="12.42578125" customWidth="1"/>
+    <col min="165" max="165" width="12.140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:175" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:175" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>372</v>
       </c>
@@ -63958,7 +63961,7 @@
         <v>189</v>
       </c>
     </row>
-    <row r="2" spans="1:175" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:175" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>373</v>
       </c>
@@ -64482,14 +64485,14 @@
         <v>371</v>
       </c>
     </row>
-    <row r="3" spans="1:175" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:175" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>374</v>
       </c>
       <c r="R3" s="1"/>
       <c r="CA3" s="1"/>
     </row>
-    <row r="4" spans="1:175" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:175" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>375</v>
       </c>
@@ -65013,7 +65016,7 @@
         <v>371</v>
       </c>
     </row>
-    <row r="5" spans="1:175" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:175" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>376</v>
       </c>
@@ -65537,7 +65540,7 @@
         <v>371</v>
       </c>
     </row>
-    <row r="6" spans="1:175" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:175" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>377</v>
       </c>
@@ -66061,7 +66064,7 @@
         <v>371</v>
       </c>
     </row>
-    <row r="7" spans="1:175" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:175" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>378</v>
       </c>
@@ -66585,11 +66588,11 @@
         <v>371</v>
       </c>
     </row>
-    <row r="8" spans="1:175" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:175" x14ac:dyDescent="0.25">
       <c r="R8" s="1"/>
       <c r="CA8" s="1"/>
     </row>
-    <row r="9" spans="1:175" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:175" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>198</v>
       </c>
@@ -67116,7 +67119,7 @@
         <v>197</v>
       </c>
     </row>
-    <row r="10" spans="1:175" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:175" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>199</v>
       </c>

</xml_diff>